<commit_message>
farklı klasörden okuma ve yazma hatası düzeltildi.
</commit_message>
<xml_diff>
--- a/Stok Kontrol/Eklenen.xlsx
+++ b/Stok Kontrol/Eklenen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yak\Desktop\Python\Stok Kontrol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB4FAB23-8342-46CF-8281-008B6F5A3588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB6D44DE-9187-41FC-8645-FB094F3FDCBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="329">
   <si>
     <t>BARKOD NUMARASI</t>
   </si>
@@ -594,6 +594,435 @@
   </si>
   <si>
     <t>88462400-295</t>
+  </si>
+  <si>
+    <t>89386900-17</t>
+  </si>
+  <si>
+    <t>000000000040002352</t>
+  </si>
+  <si>
+    <t>89455600-56</t>
+  </si>
+  <si>
+    <t>89456200-51</t>
+  </si>
+  <si>
+    <t>000000000040000813</t>
+  </si>
+  <si>
+    <t>89466500-1</t>
+  </si>
+  <si>
+    <t>89466500-3</t>
+  </si>
+  <si>
+    <t>89466500-4</t>
+  </si>
+  <si>
+    <t>89466500-5</t>
+  </si>
+  <si>
+    <t>89466500-6</t>
+  </si>
+  <si>
+    <t>89466500-7</t>
+  </si>
+  <si>
+    <t>89466500-8</t>
+  </si>
+  <si>
+    <t>89466500-9</t>
+  </si>
+  <si>
+    <t>89466500-2</t>
+  </si>
+  <si>
+    <t>89383600-5</t>
+  </si>
+  <si>
+    <t>000000000040002076</t>
+  </si>
+  <si>
+    <t>89383600-1</t>
+  </si>
+  <si>
+    <t>89383600-4</t>
+  </si>
+  <si>
+    <t>89383600-2</t>
+  </si>
+  <si>
+    <t>89383600-3</t>
+  </si>
+  <si>
+    <t>89383600-6</t>
+  </si>
+  <si>
+    <t>89383500-1</t>
+  </si>
+  <si>
+    <t>000000000040002080</t>
+  </si>
+  <si>
+    <t>89430500-1</t>
+  </si>
+  <si>
+    <t>000000000040000570</t>
+  </si>
+  <si>
+    <t>89386900-13</t>
+  </si>
+  <si>
+    <t>89370100-111</t>
+  </si>
+  <si>
+    <t>000000000040002152</t>
+  </si>
+  <si>
+    <t>89345800-34</t>
+  </si>
+  <si>
+    <t>000000000040002500</t>
+  </si>
+  <si>
+    <t>89465500-41</t>
+  </si>
+  <si>
+    <t>000000000040002348</t>
+  </si>
+  <si>
+    <t>89371100-262</t>
+  </si>
+  <si>
+    <t>000000000040002136</t>
+  </si>
+  <si>
+    <t>89393350-1</t>
+  </si>
+  <si>
+    <t>89468300-1</t>
+  </si>
+  <si>
+    <t>89468300-2</t>
+  </si>
+  <si>
+    <t>89468300-3</t>
+  </si>
+  <si>
+    <t>89468300-4</t>
+  </si>
+  <si>
+    <t>89468300-5</t>
+  </si>
+  <si>
+    <t>89468300-6</t>
+  </si>
+  <si>
+    <t>89468300-7</t>
+  </si>
+  <si>
+    <t>89468300-8</t>
+  </si>
+  <si>
+    <t>89389200-5</t>
+  </si>
+  <si>
+    <t>000000000040002432</t>
+  </si>
+  <si>
+    <t>89466500-10</t>
+  </si>
+  <si>
+    <t>89463300-1</t>
+  </si>
+  <si>
+    <t>000000000040002090</t>
+  </si>
+  <si>
+    <t>89463400-6</t>
+  </si>
+  <si>
+    <t>000000000040002086</t>
+  </si>
+  <si>
+    <t>89463400-9</t>
+  </si>
+  <si>
+    <t>89463400-11</t>
+  </si>
+  <si>
+    <t>89463400-15</t>
+  </si>
+  <si>
+    <t>89463400-16</t>
+  </si>
+  <si>
+    <t>89463400-18</t>
+  </si>
+  <si>
+    <t>89469800-2</t>
+  </si>
+  <si>
+    <t>000000000040002287</t>
+  </si>
+  <si>
+    <t>89369200-2070</t>
+  </si>
+  <si>
+    <t>89537800-11</t>
+  </si>
+  <si>
+    <t>000000000040002515</t>
+  </si>
+  <si>
+    <t>89466900-41</t>
+  </si>
+  <si>
+    <t>000000000040002378</t>
+  </si>
+  <si>
+    <t>89369900-71</t>
+  </si>
+  <si>
+    <t>000000000040003158</t>
+  </si>
+  <si>
+    <t>71662800-10</t>
+  </si>
+  <si>
+    <t>000000000040001143</t>
+  </si>
+  <si>
+    <t>88068300-25</t>
+  </si>
+  <si>
+    <t>000000000040002102</t>
+  </si>
+  <si>
+    <t>74031100-32</t>
+  </si>
+  <si>
+    <t>000000000040001775</t>
+  </si>
+  <si>
+    <t>88756400-2</t>
+  </si>
+  <si>
+    <t>000000000040001414</t>
+  </si>
+  <si>
+    <t>84744800-8</t>
+  </si>
+  <si>
+    <t>000000000040001427</t>
+  </si>
+  <si>
+    <t>74031100-33</t>
+  </si>
+  <si>
+    <t>88756400-3</t>
+  </si>
+  <si>
+    <t>89505000-8</t>
+  </si>
+  <si>
+    <t>000000000040001638</t>
+  </si>
+  <si>
+    <t>81219200-3</t>
+  </si>
+  <si>
+    <t>000000000040001674</t>
+  </si>
+  <si>
+    <t>74039600-3</t>
+  </si>
+  <si>
+    <t>000000000040000936</t>
+  </si>
+  <si>
+    <t>74031100-34</t>
+  </si>
+  <si>
+    <t>74031100-35</t>
+  </si>
+  <si>
+    <t>89498500-43</t>
+  </si>
+  <si>
+    <t>000000000040001639</t>
+  </si>
+  <si>
+    <t>88068300-26</t>
+  </si>
+  <si>
+    <t>69592500-15</t>
+  </si>
+  <si>
+    <t>000000000040001256</t>
+  </si>
+  <si>
+    <t>69592500-16</t>
+  </si>
+  <si>
+    <t>89523100-2</t>
+  </si>
+  <si>
+    <t>000000000040000664</t>
+  </si>
+  <si>
+    <t>89354200-2</t>
+  </si>
+  <si>
+    <t>000000000040001037</t>
+  </si>
+  <si>
+    <t>89523100-3</t>
+  </si>
+  <si>
+    <t>89523100-4</t>
+  </si>
+  <si>
+    <t>89495300-2</t>
+  </si>
+  <si>
+    <t>000000000040000770</t>
+  </si>
+  <si>
+    <t>89523100-5</t>
+  </si>
+  <si>
+    <t>88756400-4</t>
+  </si>
+  <si>
+    <t>89407600-28</t>
+  </si>
+  <si>
+    <t>000000000040001118</t>
+  </si>
+  <si>
+    <t>87821500-2</t>
+  </si>
+  <si>
+    <t>000000000040002114</t>
+  </si>
+  <si>
+    <t>89354200-3</t>
+  </si>
+  <si>
+    <t>69592500-17</t>
+  </si>
+  <si>
+    <t>69592500-18</t>
+  </si>
+  <si>
+    <t>69592500-19</t>
+  </si>
+  <si>
+    <t>69592500-20</t>
+  </si>
+  <si>
+    <t>87831100-2</t>
+  </si>
+  <si>
+    <t>000000000040002106</t>
+  </si>
+  <si>
+    <t>87831100-3</t>
+  </si>
+  <si>
+    <t>81154000-64</t>
+  </si>
+  <si>
+    <t>000000000040002129</t>
+  </si>
+  <si>
+    <t>88065200-2</t>
+  </si>
+  <si>
+    <t>000000000040002108</t>
+  </si>
+  <si>
+    <t>73257300-69</t>
+  </si>
+  <si>
+    <t>000000000040001449</t>
+  </si>
+  <si>
+    <t>88579300-193</t>
+  </si>
+  <si>
+    <t>000000000040000939</t>
+  </si>
+  <si>
+    <t>89250400-29</t>
+  </si>
+  <si>
+    <t>000000000040001869</t>
+  </si>
+  <si>
+    <t>69592500-21</t>
+  </si>
+  <si>
+    <t>88065200-3</t>
+  </si>
+  <si>
+    <t>84379300-113</t>
+  </si>
+  <si>
+    <t>000000000040000906</t>
+  </si>
+  <si>
+    <t>89286600-15</t>
+  </si>
+  <si>
+    <t>000000000040001386</t>
+  </si>
+  <si>
+    <t>81217900-7</t>
+  </si>
+  <si>
+    <t>000000000040002116</t>
+  </si>
+  <si>
+    <t>87822800-2</t>
+  </si>
+  <si>
+    <t>000000000040002089</t>
+  </si>
+  <si>
+    <t>89343100-3</t>
+  </si>
+  <si>
+    <t>000000000040001008</t>
+  </si>
+  <si>
+    <t>89490500-15</t>
+  </si>
+  <si>
+    <t>000000000040001404</t>
+  </si>
+  <si>
+    <t>88065200-4</t>
+  </si>
+  <si>
+    <t>88065200-5</t>
+  </si>
+  <si>
+    <t>89398500-109</t>
+  </si>
+  <si>
+    <t>000000000040000775</t>
+  </si>
+  <si>
+    <t>89409300-2</t>
+  </si>
+  <si>
+    <t>000000000040001149</t>
+  </si>
+  <si>
+    <t>89464800-13</t>
   </si>
 </sst>
 </file>
@@ -617,7 +1046,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -625,17 +1054,39 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -656,8 +1107,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{25C5C167-F782-4D50-9FF8-811AA4D4B559}" name="EKLENEN" displayName="EKLENEN" ref="A1:E131" totalsRowShown="0">
-  <autoFilter ref="A1:E131" xr:uid="{25C5C167-F782-4D50-9FF8-811AA4D4B559}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{25C5C167-F782-4D50-9FF8-811AA4D4B559}" name="EKLENEN" displayName="EKLENEN" ref="A1:E229" totalsRowShown="0">
+  <autoFilter ref="A1:E229" xr:uid="{25C5C167-F782-4D50-9FF8-811AA4D4B559}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{C7FC6704-65BD-4F1E-AB57-95E929157E58}" name="BARKOD NUMARASI"/>
     <tableColumn id="2" xr3:uid="{BD785338-7565-42D3-ADE5-4B20FE7C87B3}" name="ÜRÜN KODU / ÜRÜN TANIMI"/>
@@ -932,12 +1383,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E131"/>
+  <dimension ref="A1:E229"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
     <col min="2" max="2" width="28.5703125" customWidth="1"/>
     <col min="3" max="3" width="10.140625" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -3141,6 +3593,1606 @@
       </c>
       <c r="E131" s="2">
         <v>46126</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>186</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C132">
+        <v>7500</v>
+      </c>
+      <c r="D132" t="s">
+        <v>6</v>
+      </c>
+      <c r="E132" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>188</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C133" s="1">
+        <v>5586</v>
+      </c>
+      <c r="E133" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>189</v>
+      </c>
+      <c r="B134" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="C134" s="1">
+        <v>5586</v>
+      </c>
+      <c r="E134" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>191</v>
+      </c>
+      <c r="B135">
+        <v>40002466</v>
+      </c>
+      <c r="C135">
+        <v>68000</v>
+      </c>
+      <c r="E135" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>192</v>
+      </c>
+      <c r="B136">
+        <v>40002466</v>
+      </c>
+      <c r="C136">
+        <v>70000</v>
+      </c>
+      <c r="E136" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>193</v>
+      </c>
+      <c r="B137">
+        <v>40002466</v>
+      </c>
+      <c r="C137">
+        <v>69000</v>
+      </c>
+      <c r="E137" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>194</v>
+      </c>
+      <c r="B138">
+        <v>40002466</v>
+      </c>
+      <c r="C138">
+        <v>62000</v>
+      </c>
+      <c r="E138" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>195</v>
+      </c>
+      <c r="B139">
+        <v>40002466</v>
+      </c>
+      <c r="C139">
+        <v>70000</v>
+      </c>
+      <c r="E139" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>196</v>
+      </c>
+      <c r="B140">
+        <v>40002466</v>
+      </c>
+      <c r="C140">
+        <v>70176</v>
+      </c>
+      <c r="E140" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>197</v>
+      </c>
+      <c r="B141">
+        <v>40002466</v>
+      </c>
+      <c r="C141">
+        <v>70000</v>
+      </c>
+      <c r="E141" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>198</v>
+      </c>
+      <c r="B142">
+        <v>40002466</v>
+      </c>
+      <c r="C142">
+        <v>70176</v>
+      </c>
+      <c r="E142" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>199</v>
+      </c>
+      <c r="B143">
+        <v>40002466</v>
+      </c>
+      <c r="C143">
+        <v>71000</v>
+      </c>
+      <c r="E143" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>200</v>
+      </c>
+      <c r="B144" t="s">
+        <v>201</v>
+      </c>
+      <c r="C144">
+        <v>2274</v>
+      </c>
+      <c r="D144" t="s">
+        <v>6</v>
+      </c>
+      <c r="E144" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>202</v>
+      </c>
+      <c r="B145" t="s">
+        <v>201</v>
+      </c>
+      <c r="C145">
+        <v>2274</v>
+      </c>
+      <c r="D145" t="s">
+        <v>6</v>
+      </c>
+      <c r="E145" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>203</v>
+      </c>
+      <c r="B146" t="s">
+        <v>201</v>
+      </c>
+      <c r="C146">
+        <v>2274</v>
+      </c>
+      <c r="D146" t="s">
+        <v>6</v>
+      </c>
+      <c r="E146" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>204</v>
+      </c>
+      <c r="B147" t="s">
+        <v>201</v>
+      </c>
+      <c r="C147">
+        <v>2274</v>
+      </c>
+      <c r="D147" t="s">
+        <v>6</v>
+      </c>
+      <c r="E147" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>205</v>
+      </c>
+      <c r="B148" t="s">
+        <v>201</v>
+      </c>
+      <c r="C148">
+        <v>2274</v>
+      </c>
+      <c r="D148" t="s">
+        <v>6</v>
+      </c>
+      <c r="E148" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>206</v>
+      </c>
+      <c r="B149" t="s">
+        <v>201</v>
+      </c>
+      <c r="C149">
+        <v>2274</v>
+      </c>
+      <c r="D149" t="s">
+        <v>6</v>
+      </c>
+      <c r="E149" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>207</v>
+      </c>
+      <c r="B150" t="s">
+        <v>208</v>
+      </c>
+      <c r="C150">
+        <v>2216</v>
+      </c>
+      <c r="D150" t="s">
+        <v>6</v>
+      </c>
+      <c r="E150" s="2">
+        <v>46126</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>209</v>
+      </c>
+      <c r="B151" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="C151">
+        <v>35009</v>
+      </c>
+      <c r="D151" t="s">
+        <v>6</v>
+      </c>
+      <c r="E151" s="2">
+        <v>46127</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>211</v>
+      </c>
+      <c r="B152" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C152">
+        <v>15000</v>
+      </c>
+      <c r="D152" t="s">
+        <v>6</v>
+      </c>
+      <c r="E152" s="2">
+        <v>46127</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>212</v>
+      </c>
+      <c r="B153" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="C153">
+        <v>540</v>
+      </c>
+      <c r="D153" t="s">
+        <v>6</v>
+      </c>
+      <c r="E153" s="2">
+        <v>46128</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>214</v>
+      </c>
+      <c r="B154" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C154">
+        <v>17550</v>
+      </c>
+      <c r="D154" t="s">
+        <v>6</v>
+      </c>
+      <c r="E154" s="2">
+        <v>46128</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>216</v>
+      </c>
+      <c r="B155" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="C155">
+        <v>6400</v>
+      </c>
+      <c r="D155" t="s">
+        <v>6</v>
+      </c>
+      <c r="E155" s="2">
+        <v>46128</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>218</v>
+      </c>
+      <c r="B156" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C156">
+        <v>34557</v>
+      </c>
+      <c r="D156" t="s">
+        <v>6</v>
+      </c>
+      <c r="E156" s="2">
+        <v>46128</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>220</v>
+      </c>
+      <c r="B157">
+        <v>45018489</v>
+      </c>
+      <c r="C157">
+        <v>426</v>
+      </c>
+      <c r="E157" s="2">
+        <v>46129</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>221</v>
+      </c>
+      <c r="B158">
+        <v>40003268</v>
+      </c>
+      <c r="C158">
+        <v>9100</v>
+      </c>
+      <c r="E158" s="2">
+        <v>46122</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>222</v>
+      </c>
+      <c r="B159">
+        <v>40003268</v>
+      </c>
+      <c r="C159">
+        <v>9200</v>
+      </c>
+      <c r="E159" s="2">
+        <v>46122</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>223</v>
+      </c>
+      <c r="B160">
+        <v>40003268</v>
+      </c>
+      <c r="C160">
+        <v>9250</v>
+      </c>
+      <c r="E160" s="2">
+        <v>46122</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>224</v>
+      </c>
+      <c r="B161">
+        <v>40003268</v>
+      </c>
+      <c r="C161">
+        <v>9200</v>
+      </c>
+      <c r="E161" s="2">
+        <v>46122</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>225</v>
+      </c>
+      <c r="B162">
+        <v>40003268</v>
+      </c>
+      <c r="C162">
+        <v>9100</v>
+      </c>
+      <c r="E162" s="2">
+        <v>46122</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>226</v>
+      </c>
+      <c r="B163">
+        <v>40003268</v>
+      </c>
+      <c r="C163">
+        <v>9200</v>
+      </c>
+      <c r="E163" s="2">
+        <v>46122</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>227</v>
+      </c>
+      <c r="B164">
+        <v>40003268</v>
+      </c>
+      <c r="C164">
+        <v>9300</v>
+      </c>
+      <c r="E164" s="2">
+        <v>46122</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>228</v>
+      </c>
+      <c r="B165">
+        <v>40003268</v>
+      </c>
+      <c r="C165">
+        <v>9200</v>
+      </c>
+      <c r="E165" s="2">
+        <v>46122</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>229</v>
+      </c>
+      <c r="B166" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="C166">
+        <v>6110</v>
+      </c>
+      <c r="D166" t="s">
+        <v>6</v>
+      </c>
+      <c r="E166" s="2">
+        <v>46129</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>231</v>
+      </c>
+      <c r="B167">
+        <v>40002466</v>
+      </c>
+      <c r="C167">
+        <v>70176</v>
+      </c>
+      <c r="E167" s="2">
+        <v>46132</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>232</v>
+      </c>
+      <c r="B168" t="s">
+        <v>233</v>
+      </c>
+      <c r="C168">
+        <v>16890</v>
+      </c>
+      <c r="D168" t="s">
+        <v>6</v>
+      </c>
+      <c r="E168" s="2">
+        <v>46132</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>234</v>
+      </c>
+      <c r="B169" t="s">
+        <v>235</v>
+      </c>
+      <c r="C169">
+        <v>5783</v>
+      </c>
+      <c r="D169" t="s">
+        <v>6</v>
+      </c>
+      <c r="E169" s="2">
+        <v>46132</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>236</v>
+      </c>
+      <c r="B170" t="s">
+        <v>235</v>
+      </c>
+      <c r="C170">
+        <v>5783</v>
+      </c>
+      <c r="D170" t="s">
+        <v>6</v>
+      </c>
+      <c r="E170" s="2">
+        <v>46132</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>237</v>
+      </c>
+      <c r="B171" t="s">
+        <v>235</v>
+      </c>
+      <c r="C171">
+        <v>5783</v>
+      </c>
+      <c r="D171" t="s">
+        <v>6</v>
+      </c>
+      <c r="E171" s="2">
+        <v>46132</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>238</v>
+      </c>
+      <c r="B172" t="s">
+        <v>235</v>
+      </c>
+      <c r="C172">
+        <v>5783</v>
+      </c>
+      <c r="D172" t="s">
+        <v>6</v>
+      </c>
+      <c r="E172" s="2">
+        <v>46132</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>239</v>
+      </c>
+      <c r="B173" t="s">
+        <v>235</v>
+      </c>
+      <c r="C173">
+        <v>5783</v>
+      </c>
+      <c r="D173" t="s">
+        <v>6</v>
+      </c>
+      <c r="E173" s="2">
+        <v>46132</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>240</v>
+      </c>
+      <c r="B174" t="s">
+        <v>235</v>
+      </c>
+      <c r="C174">
+        <v>5783</v>
+      </c>
+      <c r="D174" t="s">
+        <v>6</v>
+      </c>
+      <c r="E174" s="2">
+        <v>46132</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>241</v>
+      </c>
+      <c r="B175" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="C175">
+        <v>2400</v>
+      </c>
+      <c r="D175" t="s">
+        <v>6</v>
+      </c>
+      <c r="E175" s="2">
+        <v>46132</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>243</v>
+      </c>
+      <c r="B176" t="s">
+        <v>119</v>
+      </c>
+      <c r="C176">
+        <v>1532</v>
+      </c>
+      <c r="E176" s="2">
+        <v>46132</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>244</v>
+      </c>
+      <c r="B177" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="C177">
+        <v>3100</v>
+      </c>
+      <c r="D177" t="s">
+        <v>6</v>
+      </c>
+      <c r="E177" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A178" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="B178" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="C178">
+        <v>3100</v>
+      </c>
+      <c r="D178" t="s">
+        <v>6</v>
+      </c>
+      <c r="E178" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A179" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="B179" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="C179">
+        <v>110527</v>
+      </c>
+      <c r="D179" t="s">
+        <v>6</v>
+      </c>
+      <c r="E179" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A180" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="B180" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="C180">
+        <v>14382</v>
+      </c>
+      <c r="D180" t="s">
+        <v>6</v>
+      </c>
+      <c r="E180" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>252</v>
+      </c>
+      <c r="B181" t="s">
+        <v>253</v>
+      </c>
+      <c r="C181">
+        <v>23945</v>
+      </c>
+      <c r="D181" t="s">
+        <v>6</v>
+      </c>
+      <c r="E181" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>254</v>
+      </c>
+      <c r="B182" t="s">
+        <v>255</v>
+      </c>
+      <c r="C182">
+        <v>4361</v>
+      </c>
+      <c r="D182" t="s">
+        <v>6</v>
+      </c>
+      <c r="E182" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>256</v>
+      </c>
+      <c r="B183" t="s">
+        <v>257</v>
+      </c>
+      <c r="C183">
+        <v>4553</v>
+      </c>
+      <c r="D183" t="s">
+        <v>6</v>
+      </c>
+      <c r="E183" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>258</v>
+      </c>
+      <c r="B184" t="s">
+        <v>259</v>
+      </c>
+      <c r="C184">
+        <v>3820</v>
+      </c>
+      <c r="D184" t="s">
+        <v>6</v>
+      </c>
+      <c r="E184" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>260</v>
+      </c>
+      <c r="B185" t="s">
+        <v>255</v>
+      </c>
+      <c r="C185">
+        <v>4425</v>
+      </c>
+      <c r="D185" t="s">
+        <v>6</v>
+      </c>
+      <c r="E185" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>261</v>
+      </c>
+      <c r="B186" t="s">
+        <v>257</v>
+      </c>
+      <c r="C186">
+        <v>4425</v>
+      </c>
+      <c r="D186" t="s">
+        <v>6</v>
+      </c>
+      <c r="E186" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
+        <v>262</v>
+      </c>
+      <c r="B187" t="s">
+        <v>263</v>
+      </c>
+      <c r="C187">
+        <v>6128</v>
+      </c>
+      <c r="D187" t="s">
+        <v>6</v>
+      </c>
+      <c r="E187" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>264</v>
+      </c>
+      <c r="B188" t="s">
+        <v>265</v>
+      </c>
+      <c r="C188">
+        <v>3443</v>
+      </c>
+      <c r="D188" t="s">
+        <v>6</v>
+      </c>
+      <c r="E188" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>266</v>
+      </c>
+      <c r="B189" t="s">
+        <v>267</v>
+      </c>
+      <c r="C189">
+        <v>2306</v>
+      </c>
+      <c r="D189" t="s">
+        <v>6</v>
+      </c>
+      <c r="E189" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>268</v>
+      </c>
+      <c r="B190" t="s">
+        <v>255</v>
+      </c>
+      <c r="C190">
+        <v>4425</v>
+      </c>
+      <c r="D190" t="s">
+        <v>6</v>
+      </c>
+      <c r="E190" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>269</v>
+      </c>
+      <c r="B191" t="s">
+        <v>255</v>
+      </c>
+      <c r="C191">
+        <v>5067</v>
+      </c>
+      <c r="D191" t="s">
+        <v>6</v>
+      </c>
+      <c r="E191" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>270</v>
+      </c>
+      <c r="B192" t="s">
+        <v>271</v>
+      </c>
+      <c r="C192">
+        <v>8360</v>
+      </c>
+      <c r="D192" t="s">
+        <v>6</v>
+      </c>
+      <c r="E192" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>272</v>
+      </c>
+      <c r="B193" t="s">
+        <v>253</v>
+      </c>
+      <c r="C193">
+        <v>4018</v>
+      </c>
+      <c r="D193" t="s">
+        <v>6</v>
+      </c>
+      <c r="E193" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
+        <v>273</v>
+      </c>
+      <c r="B194" t="s">
+        <v>274</v>
+      </c>
+      <c r="C194">
+        <v>6731</v>
+      </c>
+      <c r="D194" t="s">
+        <v>6</v>
+      </c>
+      <c r="E194" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
+        <v>275</v>
+      </c>
+      <c r="B195" t="s">
+        <v>274</v>
+      </c>
+      <c r="C195">
+        <v>6436</v>
+      </c>
+      <c r="D195" t="s">
+        <v>6</v>
+      </c>
+      <c r="E195" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>276</v>
+      </c>
+      <c r="B196" t="s">
+        <v>277</v>
+      </c>
+      <c r="C196">
+        <v>3362</v>
+      </c>
+      <c r="D196" t="s">
+        <v>6</v>
+      </c>
+      <c r="E196" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>278</v>
+      </c>
+      <c r="B197" t="s">
+        <v>279</v>
+      </c>
+      <c r="C197">
+        <v>3362</v>
+      </c>
+      <c r="D197" t="s">
+        <v>6</v>
+      </c>
+      <c r="E197" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>280</v>
+      </c>
+      <c r="B198" t="s">
+        <v>277</v>
+      </c>
+      <c r="C198">
+        <v>3362</v>
+      </c>
+      <c r="D198" t="s">
+        <v>6</v>
+      </c>
+      <c r="E198" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
+        <v>281</v>
+      </c>
+      <c r="B199" t="s">
+        <v>277</v>
+      </c>
+      <c r="C199">
+        <v>3362</v>
+      </c>
+      <c r="D199" t="s">
+        <v>6</v>
+      </c>
+      <c r="E199" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>282</v>
+      </c>
+      <c r="B200" t="s">
+        <v>283</v>
+      </c>
+      <c r="C200">
+        <v>3362</v>
+      </c>
+      <c r="D200" t="s">
+        <v>6</v>
+      </c>
+      <c r="E200" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>284</v>
+      </c>
+      <c r="B201" t="s">
+        <v>277</v>
+      </c>
+      <c r="C201">
+        <v>3362</v>
+      </c>
+      <c r="D201" t="s">
+        <v>6</v>
+      </c>
+      <c r="E201" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>285</v>
+      </c>
+      <c r="B202" t="s">
+        <v>257</v>
+      </c>
+      <c r="C202">
+        <v>2277</v>
+      </c>
+      <c r="D202" t="s">
+        <v>6</v>
+      </c>
+      <c r="E202" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>286</v>
+      </c>
+      <c r="B203" t="s">
+        <v>287</v>
+      </c>
+      <c r="C203">
+        <v>6926</v>
+      </c>
+      <c r="D203" t="s">
+        <v>6</v>
+      </c>
+      <c r="E203" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>288</v>
+      </c>
+      <c r="B204" t="s">
+        <v>289</v>
+      </c>
+      <c r="C204">
+        <v>2424</v>
+      </c>
+      <c r="D204" t="s">
+        <v>6</v>
+      </c>
+      <c r="E204" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
+        <v>290</v>
+      </c>
+      <c r="B205" t="s">
+        <v>279</v>
+      </c>
+      <c r="C205">
+        <v>2944</v>
+      </c>
+      <c r="D205" t="s">
+        <v>6</v>
+      </c>
+      <c r="E205" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A206" t="s">
+        <v>291</v>
+      </c>
+      <c r="B206" t="s">
+        <v>274</v>
+      </c>
+      <c r="C206">
+        <v>7204</v>
+      </c>
+      <c r="D206" t="s">
+        <v>6</v>
+      </c>
+      <c r="E206" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A207" t="s">
+        <v>292</v>
+      </c>
+      <c r="B207" t="s">
+        <v>274</v>
+      </c>
+      <c r="C207">
+        <v>6731</v>
+      </c>
+      <c r="D207" t="s">
+        <v>6</v>
+      </c>
+      <c r="E207" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
+        <v>293</v>
+      </c>
+      <c r="B208" t="s">
+        <v>274</v>
+      </c>
+      <c r="C208">
+        <v>6926</v>
+      </c>
+      <c r="D208" t="s">
+        <v>6</v>
+      </c>
+      <c r="E208" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
+        <v>294</v>
+      </c>
+      <c r="B209" t="s">
+        <v>274</v>
+      </c>
+      <c r="C209">
+        <v>6628</v>
+      </c>
+      <c r="D209" t="s">
+        <v>6</v>
+      </c>
+      <c r="E209" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
+        <v>295</v>
+      </c>
+      <c r="B210" t="s">
+        <v>296</v>
+      </c>
+      <c r="C210">
+        <v>3276</v>
+      </c>
+      <c r="D210" t="s">
+        <v>6</v>
+      </c>
+      <c r="E210" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A211" t="s">
+        <v>297</v>
+      </c>
+      <c r="B211" t="s">
+        <v>296</v>
+      </c>
+      <c r="C211">
+        <v>2982</v>
+      </c>
+      <c r="D211" t="s">
+        <v>6</v>
+      </c>
+      <c r="E211" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A212" t="s">
+        <v>298</v>
+      </c>
+      <c r="B212" t="s">
+        <v>299</v>
+      </c>
+      <c r="C212">
+        <v>2738</v>
+      </c>
+      <c r="D212" t="s">
+        <v>6</v>
+      </c>
+      <c r="E212" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A213" t="s">
+        <v>300</v>
+      </c>
+      <c r="B213" t="s">
+        <v>301</v>
+      </c>
+      <c r="C213">
+        <v>3236</v>
+      </c>
+      <c r="D213" t="s">
+        <v>6</v>
+      </c>
+      <c r="E213" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A214" t="s">
+        <v>302</v>
+      </c>
+      <c r="B214" t="s">
+        <v>303</v>
+      </c>
+      <c r="C214">
+        <v>981</v>
+      </c>
+      <c r="D214" t="s">
+        <v>6</v>
+      </c>
+      <c r="E214" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A215" t="s">
+        <v>304</v>
+      </c>
+      <c r="B215" t="s">
+        <v>305</v>
+      </c>
+      <c r="C215">
+        <v>692</v>
+      </c>
+      <c r="D215" t="s">
+        <v>6</v>
+      </c>
+      <c r="E215" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
+        <v>306</v>
+      </c>
+      <c r="B216" t="s">
+        <v>307</v>
+      </c>
+      <c r="C216">
+        <v>3276</v>
+      </c>
+      <c r="D216" t="s">
+        <v>6</v>
+      </c>
+      <c r="E216" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
+        <v>308</v>
+      </c>
+      <c r="B217" t="s">
+        <v>274</v>
+      </c>
+      <c r="C217">
+        <v>6926</v>
+      </c>
+      <c r="D217" t="s">
+        <v>6</v>
+      </c>
+      <c r="E217" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A218" t="s">
+        <v>309</v>
+      </c>
+      <c r="B218" t="s">
+        <v>301</v>
+      </c>
+      <c r="C218">
+        <v>1983</v>
+      </c>
+      <c r="D218" t="s">
+        <v>6</v>
+      </c>
+      <c r="E218" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
+        <v>310</v>
+      </c>
+      <c r="B219" t="s">
+        <v>311</v>
+      </c>
+      <c r="C219">
+        <v>1692</v>
+      </c>
+      <c r="D219" t="s">
+        <v>6</v>
+      </c>
+      <c r="E219" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
+        <v>312</v>
+      </c>
+      <c r="B220" t="s">
+        <v>313</v>
+      </c>
+      <c r="C220">
+        <v>2943</v>
+      </c>
+      <c r="D220" t="s">
+        <v>6</v>
+      </c>
+      <c r="E220" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
+        <v>314</v>
+      </c>
+      <c r="B221" t="s">
+        <v>315</v>
+      </c>
+      <c r="C221">
+        <v>1176</v>
+      </c>
+      <c r="D221" t="s">
+        <v>6</v>
+      </c>
+      <c r="E221" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A222" t="s">
+        <v>316</v>
+      </c>
+      <c r="B222" t="s">
+        <v>317</v>
+      </c>
+      <c r="C222">
+        <v>4429</v>
+      </c>
+      <c r="D222" t="s">
+        <v>6</v>
+      </c>
+      <c r="E222" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A223" t="s">
+        <v>318</v>
+      </c>
+      <c r="B223" t="s">
+        <v>319</v>
+      </c>
+      <c r="C223">
+        <v>6727</v>
+      </c>
+      <c r="D223" t="s">
+        <v>6</v>
+      </c>
+      <c r="E223" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
+        <v>320</v>
+      </c>
+      <c r="B224" t="s">
+        <v>321</v>
+      </c>
+      <c r="C224">
+        <v>3450</v>
+      </c>
+      <c r="D224" t="s">
+        <v>6</v>
+      </c>
+      <c r="E224" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
+        <v>322</v>
+      </c>
+      <c r="B225" t="s">
+        <v>301</v>
+      </c>
+      <c r="C225">
+        <v>3097</v>
+      </c>
+      <c r="D225" t="s">
+        <v>6</v>
+      </c>
+      <c r="E225" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A226" t="s">
+        <v>323</v>
+      </c>
+      <c r="B226" t="s">
+        <v>301</v>
+      </c>
+      <c r="C226">
+        <v>3236</v>
+      </c>
+      <c r="D226" t="s">
+        <v>6</v>
+      </c>
+      <c r="E226" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A227" t="s">
+        <v>324</v>
+      </c>
+      <c r="B227" t="s">
+        <v>325</v>
+      </c>
+      <c r="C227">
+        <v>2092</v>
+      </c>
+      <c r="D227" t="s">
+        <v>6</v>
+      </c>
+      <c r="E227" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A228" t="s">
+        <v>326</v>
+      </c>
+      <c r="B228" t="s">
+        <v>327</v>
+      </c>
+      <c r="C228">
+        <v>3715</v>
+      </c>
+      <c r="D228" t="s">
+        <v>6</v>
+      </c>
+      <c r="E228" s="2">
+        <v>46133</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A229" t="s">
+        <v>328</v>
+      </c>
+      <c r="B229" t="s">
+        <v>235</v>
+      </c>
+      <c r="C229">
+        <v>3532</v>
+      </c>
+      <c r="D229" t="s">
+        <v>6</v>
+      </c>
+      <c r="E229" s="2">
+        <v>46133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
parça sepet iüretim ve tüketim takibi yapılabilir
</commit_message>
<xml_diff>
--- a/Stok Kontrol/Eklenen.xlsx
+++ b/Stok Kontrol/Eklenen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yak\Desktop\Python\Stok Kontrol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB6D44DE-9187-41FC-8645-FB094F3FDCBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7D12C2A-EFA0-4636-9C67-69D7F94E653C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="724" uniqueCount="364">
   <si>
     <t>BARKOD NUMARASI</t>
   </si>
@@ -1023,6 +1023,111 @@
   </si>
   <si>
     <t>89464800-13</t>
+  </si>
+  <si>
+    <t>89470700-21</t>
+  </si>
+  <si>
+    <t>000000000040002728</t>
+  </si>
+  <si>
+    <t>89424600-13</t>
+  </si>
+  <si>
+    <t>000000000040003594</t>
+  </si>
+  <si>
+    <t>89424600-9</t>
+  </si>
+  <si>
+    <t>89424600-8</t>
+  </si>
+  <si>
+    <t>89424600-2</t>
+  </si>
+  <si>
+    <t>89424600-12</t>
+  </si>
+  <si>
+    <t>89424600-3</t>
+  </si>
+  <si>
+    <t>89424400-5</t>
+  </si>
+  <si>
+    <t>000000000040003506</t>
+  </si>
+  <si>
+    <t>89424400-12</t>
+  </si>
+  <si>
+    <t>89424400-9</t>
+  </si>
+  <si>
+    <t>89424400-11</t>
+  </si>
+  <si>
+    <t>89424400-3</t>
+  </si>
+  <si>
+    <t>89424400-7</t>
+  </si>
+  <si>
+    <t>89424800-14</t>
+  </si>
+  <si>
+    <t>000000000040000836</t>
+  </si>
+  <si>
+    <t>89424800-20</t>
+  </si>
+  <si>
+    <t>89424800-18</t>
+  </si>
+  <si>
+    <t>89424800-16</t>
+  </si>
+  <si>
+    <t>89424800-11</t>
+  </si>
+  <si>
+    <t>89424800-13</t>
+  </si>
+  <si>
+    <t>89424800-7</t>
+  </si>
+  <si>
+    <t>89424800-2</t>
+  </si>
+  <si>
+    <t>89424800-10</t>
+  </si>
+  <si>
+    <t>89424800-15</t>
+  </si>
+  <si>
+    <t>89424800-17</t>
+  </si>
+  <si>
+    <t>89424800-4</t>
+  </si>
+  <si>
+    <t>89424200-2</t>
+  </si>
+  <si>
+    <t>000000000040000842</t>
+  </si>
+  <si>
+    <t>89462900-1</t>
+  </si>
+  <si>
+    <t>000000000040002074</t>
+  </si>
+  <si>
+    <t>000000000040002442</t>
+  </si>
+  <si>
+    <t>89486000-20</t>
   </si>
 </sst>
 </file>
@@ -1107,8 +1212,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{25C5C167-F782-4D50-9FF8-811AA4D4B559}" name="EKLENEN" displayName="EKLENEN" ref="A1:E229" totalsRowShown="0">
-  <autoFilter ref="A1:E229" xr:uid="{25C5C167-F782-4D50-9FF8-811AA4D4B559}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{25C5C167-F782-4D50-9FF8-811AA4D4B559}" name="EKLENEN" displayName="EKLENEN" ref="A1:E257" totalsRowShown="0">
+  <autoFilter ref="A1:E257" xr:uid="{25C5C167-F782-4D50-9FF8-811AA4D4B559}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{C7FC6704-65BD-4F1E-AB57-95E929157E58}" name="BARKOD NUMARASI"/>
     <tableColumn id="2" xr3:uid="{BD785338-7565-42D3-ADE5-4B20FE7C87B3}" name="ÜRÜN KODU / ÜRÜN TANIMI"/>
@@ -1383,7 +1488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E229"/>
+  <dimension ref="A1:E257"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -5195,6 +5300,482 @@
         <v>46133</v>
       </c>
     </row>
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A230" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="B230" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="C230">
+        <v>7110</v>
+      </c>
+      <c r="D230" t="s">
+        <v>6</v>
+      </c>
+      <c r="E230" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A231" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="B231" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="C231">
+        <v>4522</v>
+      </c>
+      <c r="D231" t="s">
+        <v>6</v>
+      </c>
+      <c r="E231" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A232" t="s">
+        <v>333</v>
+      </c>
+      <c r="B232" t="s">
+        <v>332</v>
+      </c>
+      <c r="C232">
+        <v>4522</v>
+      </c>
+      <c r="D232" t="s">
+        <v>6</v>
+      </c>
+      <c r="E232" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A233" t="s">
+        <v>334</v>
+      </c>
+      <c r="B233" t="s">
+        <v>332</v>
+      </c>
+      <c r="C233">
+        <v>4522</v>
+      </c>
+      <c r="D233" t="s">
+        <v>6</v>
+      </c>
+      <c r="E233" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A234" t="s">
+        <v>335</v>
+      </c>
+      <c r="B234" t="s">
+        <v>332</v>
+      </c>
+      <c r="C234">
+        <v>4522</v>
+      </c>
+      <c r="D234" t="s">
+        <v>6</v>
+      </c>
+      <c r="E234" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A235" t="s">
+        <v>336</v>
+      </c>
+      <c r="B235" t="s">
+        <v>332</v>
+      </c>
+      <c r="C235">
+        <v>4522</v>
+      </c>
+      <c r="D235" t="s">
+        <v>6</v>
+      </c>
+      <c r="E235" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A236" t="s">
+        <v>337</v>
+      </c>
+      <c r="B236" t="s">
+        <v>332</v>
+      </c>
+      <c r="C236">
+        <v>4522</v>
+      </c>
+      <c r="D236" t="s">
+        <v>6</v>
+      </c>
+      <c r="E236" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A237" t="s">
+        <v>338</v>
+      </c>
+      <c r="B237" t="s">
+        <v>339</v>
+      </c>
+      <c r="C237">
+        <v>4452</v>
+      </c>
+      <c r="D237" t="s">
+        <v>6</v>
+      </c>
+      <c r="E237" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A238" t="s">
+        <v>340</v>
+      </c>
+      <c r="B238" t="s">
+        <v>339</v>
+      </c>
+      <c r="C238">
+        <v>4452</v>
+      </c>
+      <c r="D238" t="s">
+        <v>6</v>
+      </c>
+      <c r="E238" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A239" t="s">
+        <v>341</v>
+      </c>
+      <c r="B239" t="s">
+        <v>339</v>
+      </c>
+      <c r="C239">
+        <v>4452</v>
+      </c>
+      <c r="D239" t="s">
+        <v>6</v>
+      </c>
+      <c r="E239" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A240" t="s">
+        <v>342</v>
+      </c>
+      <c r="B240" t="s">
+        <v>339</v>
+      </c>
+      <c r="C240">
+        <v>4452</v>
+      </c>
+      <c r="D240" t="s">
+        <v>6</v>
+      </c>
+      <c r="E240" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A241" t="s">
+        <v>343</v>
+      </c>
+      <c r="B241" t="s">
+        <v>339</v>
+      </c>
+      <c r="C241">
+        <v>4452</v>
+      </c>
+      <c r="D241" t="s">
+        <v>6</v>
+      </c>
+      <c r="E241" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A242" t="s">
+        <v>344</v>
+      </c>
+      <c r="B242" t="s">
+        <v>339</v>
+      </c>
+      <c r="C242">
+        <v>4452</v>
+      </c>
+      <c r="D242" t="s">
+        <v>6</v>
+      </c>
+      <c r="E242" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A243" t="s">
+        <v>345</v>
+      </c>
+      <c r="B243" t="s">
+        <v>346</v>
+      </c>
+      <c r="C243">
+        <v>4582</v>
+      </c>
+      <c r="D243" t="s">
+        <v>6</v>
+      </c>
+      <c r="E243" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A244" t="s">
+        <v>347</v>
+      </c>
+      <c r="B244" t="s">
+        <v>346</v>
+      </c>
+      <c r="C244">
+        <v>4582</v>
+      </c>
+      <c r="D244" t="s">
+        <v>6</v>
+      </c>
+      <c r="E244" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A245" t="s">
+        <v>348</v>
+      </c>
+      <c r="B245" t="s">
+        <v>346</v>
+      </c>
+      <c r="C245">
+        <v>4582</v>
+      </c>
+      <c r="D245" t="s">
+        <v>6</v>
+      </c>
+      <c r="E245" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A246" t="s">
+        <v>349</v>
+      </c>
+      <c r="B246" t="s">
+        <v>346</v>
+      </c>
+      <c r="C246">
+        <v>4582</v>
+      </c>
+      <c r="D246" t="s">
+        <v>6</v>
+      </c>
+      <c r="E246" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A247" t="s">
+        <v>350</v>
+      </c>
+      <c r="B247" t="s">
+        <v>346</v>
+      </c>
+      <c r="C247">
+        <v>4582</v>
+      </c>
+      <c r="D247" t="s">
+        <v>6</v>
+      </c>
+      <c r="E247" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A248" t="s">
+        <v>351</v>
+      </c>
+      <c r="B248" t="s">
+        <v>346</v>
+      </c>
+      <c r="C248">
+        <v>4582</v>
+      </c>
+      <c r="D248" t="s">
+        <v>6</v>
+      </c>
+      <c r="E248" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A249" t="s">
+        <v>352</v>
+      </c>
+      <c r="B249" t="s">
+        <v>346</v>
+      </c>
+      <c r="C249">
+        <v>4582</v>
+      </c>
+      <c r="D249" t="s">
+        <v>6</v>
+      </c>
+      <c r="E249" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A250" t="s">
+        <v>353</v>
+      </c>
+      <c r="B250" t="s">
+        <v>346</v>
+      </c>
+      <c r="C250">
+        <v>4582</v>
+      </c>
+      <c r="D250" t="s">
+        <v>6</v>
+      </c>
+      <c r="E250" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A251" t="s">
+        <v>354</v>
+      </c>
+      <c r="B251" t="s">
+        <v>346</v>
+      </c>
+      <c r="C251">
+        <v>4582</v>
+      </c>
+      <c r="D251" t="s">
+        <v>6</v>
+      </c>
+      <c r="E251" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A252" t="s">
+        <v>355</v>
+      </c>
+      <c r="B252" t="s">
+        <v>346</v>
+      </c>
+      <c r="C252">
+        <v>4582</v>
+      </c>
+      <c r="D252" t="s">
+        <v>6</v>
+      </c>
+      <c r="E252" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A253" t="s">
+        <v>356</v>
+      </c>
+      <c r="B253" t="s">
+        <v>346</v>
+      </c>
+      <c r="C253">
+        <v>4582</v>
+      </c>
+      <c r="D253" t="s">
+        <v>6</v>
+      </c>
+      <c r="E253" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A254" t="s">
+        <v>357</v>
+      </c>
+      <c r="B254" t="s">
+        <v>346</v>
+      </c>
+      <c r="C254">
+        <v>4582</v>
+      </c>
+      <c r="D254" t="s">
+        <v>6</v>
+      </c>
+      <c r="E254" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A255" t="s">
+        <v>358</v>
+      </c>
+      <c r="B255" t="s">
+        <v>359</v>
+      </c>
+      <c r="C255">
+        <v>4325</v>
+      </c>
+      <c r="D255" t="s">
+        <v>6</v>
+      </c>
+      <c r="E255" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A256" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="B256" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="C256">
+        <v>8829</v>
+      </c>
+      <c r="D256" t="s">
+        <v>6</v>
+      </c>
+      <c r="E256" s="2">
+        <v>46134</v>
+      </c>
+    </row>
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A257" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="B257" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="C257">
+        <v>29350</v>
+      </c>
+      <c r="D257" t="s">
+        <v>6</v>
+      </c>
+      <c r="E257" s="2">
+        <v>46134</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Sayım stoklarında gelmeyen malzeme kodları artık geliyor.
</commit_message>
<xml_diff>
--- a/Stok Kontrol/Eklenen.xlsx
+++ b/Stok Kontrol/Eklenen.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yak\Desktop\Python\Stok Kontrol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1A8DD23-0201-4806-A1C3-6982C31DA154}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A4BE518-E882-472B-9649-A37A659428A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="33">
   <si>
     <t>BARKOD NUMARASI</t>
   </si>
@@ -81,6 +81,60 @@
   </si>
   <si>
     <t>89547700-12</t>
+  </si>
+  <si>
+    <t>89369500-19</t>
+  </si>
+  <si>
+    <t>000000000040002159</t>
+  </si>
+  <si>
+    <t>000000000040002072</t>
+  </si>
+  <si>
+    <t>89558500-3</t>
+  </si>
+  <si>
+    <t>89582400-1</t>
+  </si>
+  <si>
+    <t>89607900-201</t>
+  </si>
+  <si>
+    <t>000000000040002136</t>
+  </si>
+  <si>
+    <t>89530800-15</t>
+  </si>
+  <si>
+    <t>000000000040002444</t>
+  </si>
+  <si>
+    <t>89530800-14</t>
+  </si>
+  <si>
+    <t>89365800-20</t>
+  </si>
+  <si>
+    <t>000000000040002441</t>
+  </si>
+  <si>
+    <t>89551100-4</t>
+  </si>
+  <si>
+    <t>000000000040000825</t>
+  </si>
+  <si>
+    <t>89549400-9</t>
+  </si>
+  <si>
+    <t>000000000040002545</t>
+  </si>
+  <si>
+    <t>89584600-14</t>
+  </si>
+  <si>
+    <t>000000000040002063</t>
   </si>
 </sst>
 </file>
@@ -140,8 +194,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{25C5C167-F782-4D50-9FF8-811AA4D4B559}" name="EKLENEN" displayName="EKLENEN" ref="A1:E7" totalsRowShown="0">
-  <autoFilter ref="A1:E7" xr:uid="{25C5C167-F782-4D50-9FF8-811AA4D4B559}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{25C5C167-F782-4D50-9FF8-811AA4D4B559}" name="EKLENEN" displayName="EKLENEN" ref="A1:E17" totalsRowShown="0">
+  <autoFilter ref="A1:E17" xr:uid="{25C5C167-F782-4D50-9FF8-811AA4D4B559}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{C7FC6704-65BD-4F1E-AB57-95E929157E58}" name="BARKOD NUMARASI"/>
     <tableColumn id="2" xr3:uid="{BD785338-7565-42D3-ADE5-4B20FE7C87B3}" name="ÜRÜN KODU / ÜRÜN TANIMI"/>
@@ -416,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -544,6 +598,176 @@
         <v>46146</v>
       </c>
     </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8">
+        <v>2870</v>
+      </c>
+      <c r="D8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E8" s="2">
+        <v>46146</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9">
+        <v>2686</v>
+      </c>
+      <c r="D9" t="s">
+        <v>4</v>
+      </c>
+      <c r="E9" s="2">
+        <v>46147</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10">
+        <v>1108</v>
+      </c>
+      <c r="D10" t="s">
+        <v>4</v>
+      </c>
+      <c r="E10" s="2">
+        <v>46147</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11">
+        <v>17137</v>
+      </c>
+      <c r="D11" t="s">
+        <v>4</v>
+      </c>
+      <c r="E11" s="2">
+        <v>46147</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12">
+        <v>54310</v>
+      </c>
+      <c r="D12" t="s">
+        <v>4</v>
+      </c>
+      <c r="E12" s="2">
+        <v>46147</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13">
+        <v>45000</v>
+      </c>
+      <c r="D13" t="s">
+        <v>4</v>
+      </c>
+      <c r="E13" s="2">
+        <v>46147</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14">
+        <v>110000</v>
+      </c>
+      <c r="D14" t="s">
+        <v>4</v>
+      </c>
+      <c r="E14" s="2">
+        <v>46147</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15">
+        <v>30583</v>
+      </c>
+      <c r="D15" t="s">
+        <v>4</v>
+      </c>
+      <c r="E15" s="2">
+        <v>46147</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16">
+        <v>121520</v>
+      </c>
+      <c r="D16" t="s">
+        <v>4</v>
+      </c>
+      <c r="E16" s="2">
+        <v>46147</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17">
+        <v>4380</v>
+      </c>
+      <c r="D17" t="s">
+        <v>4</v>
+      </c>
+      <c r="E17" s="2">
+        <v>46148</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>